<commit_message>
Final commit before merging
</commit_message>
<xml_diff>
--- a/invoices/output/tracker.xlsx
+++ b/invoices/output/tracker.xlsx
@@ -2,14 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="500" windowWidth="33600" windowHeight="18980" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Invoice Tracker" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -25,14 +26,11 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <family val="2"/>
       <b val="1"/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="11"/>
+      <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -41,7 +39,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF2F5496"/>
+        <fgColor rgb="002F5496"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
     <fill>
@@ -67,16 +70,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -440,11 +444,13 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:L16"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="2"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="5"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
@@ -519,7 +525,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07 18:51</t>
+          <t>2026-06-07 19:48</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -553,29 +559,29 @@
         </is>
       </c>
       <c r="H2" s="2" t="n">
-        <v>100300</v>
+        <v>85000</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>85000</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>15300</v>
+        <v>0</v>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>AMOUNT_MISMATCH</t>
+          <t>MATCH</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Invoice amount 100300 does not match PO approved amount 85000.0. Difference: 15,300</t>
+          <t>Invoice matches PO record.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07 18:52</t>
+          <t>2026-06-07 19:48</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -609,29 +615,29 @@
         </is>
       </c>
       <c r="H3" s="2" t="n">
-        <v>49560</v>
+        <v>42000</v>
       </c>
       <c r="I3" s="2" t="n">
         <v>42000</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>7560</v>
+        <v>0</v>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>AMOUNT_MISMATCH</t>
+          <t>MATCH</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Invoice amount 49560 does not match PO approved amount 42000.0. Difference: 7,560</t>
+          <t>Invoice matches PO record.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07 18:52</t>
+          <t>2026-06-07 19:48</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -665,29 +671,29 @@
         </is>
       </c>
       <c r="H4" s="2" t="n">
-        <v>107380</v>
+        <v>91000</v>
       </c>
       <c r="I4" s="2" t="n">
         <v>91000</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>16380</v>
+        <v>0</v>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>AMOUNT_MISMATCH</t>
+          <t>MATCH</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>Invoice amount 107380 does not match PO approved amount 91000.0. Difference: 16,380</t>
+          <t>Invoice matches PO record.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07 18:52</t>
+          <t>2026-06-07 19:48</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -721,29 +727,29 @@
         </is>
       </c>
       <c r="H5" s="2" t="n">
-        <v>45430</v>
+        <v>38500</v>
       </c>
       <c r="I5" s="2" t="n">
         <v>38500</v>
       </c>
       <c r="J5" s="2" t="n">
-        <v>6930</v>
+        <v>0</v>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>AMOUNT_MISMATCH</t>
+          <t>MATCH</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>Invoice amount 45430 does not match PO approved amount 38500.0. Difference: 6,930</t>
+          <t>Invoice matches PO record.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07 18:52</t>
+          <t>2026-06-07 19:48</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -777,29 +783,29 @@
         </is>
       </c>
       <c r="H6" s="2" t="n">
-        <v>84960</v>
+        <v>72000</v>
       </c>
       <c r="I6" s="2" t="n">
         <v>72000</v>
       </c>
       <c r="J6" s="2" t="n">
-        <v>12960</v>
+        <v>0</v>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>AMOUNT_MISMATCH</t>
+          <t>MATCH</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>Invoice amount 84960 does not match PO approved amount 72000.0. Difference: 12,960</t>
+          <t>Invoice matches PO record.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07 18:52</t>
+          <t>2026-06-07 19:48</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -833,29 +839,29 @@
         </is>
       </c>
       <c r="H7" s="2" t="n">
-        <v>34810</v>
+        <v>29500</v>
       </c>
       <c r="I7" s="2" t="n">
         <v>29500</v>
       </c>
       <c r="J7" s="2" t="n">
-        <v>5310</v>
+        <v>0</v>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>AMOUNT_MISMATCH</t>
+          <t>MATCH</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>Invoice amount 34810 does not match PO approved amount 29500.0. Difference: 5,310</t>
+          <t>Invoice matches PO record.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07 18:52</t>
+          <t>2026-06-07 19:48</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -889,29 +895,29 @@
         </is>
       </c>
       <c r="H8" s="2" t="n">
-        <v>74340</v>
+        <v>63000</v>
       </c>
       <c r="I8" s="2" t="n">
         <v>63000</v>
       </c>
       <c r="J8" s="2" t="n">
-        <v>11340</v>
+        <v>0</v>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>AMOUNT_MISMATCH</t>
+          <t>MATCH</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>Invoice amount 74340 does not match PO approved amount 63000.0. Difference: 11,340</t>
+          <t>Invoice matches PO record.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07 18:52</t>
+          <t>2026-06-07 19:48</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -945,356 +951,356 @@
         </is>
       </c>
       <c r="H9" s="2" t="n">
-        <v>63720</v>
+        <v>54000</v>
       </c>
       <c r="I9" s="2" t="n">
         <v>54000</v>
       </c>
       <c r="J9" s="2" t="n">
-        <v>9720</v>
+        <v>0</v>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
+          <t>MATCH</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>Invoice matches PO record.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-07 19:48</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>INV-009.docx</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>INV-009</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Ltd</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Tata Consultancy Services Ltd</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>2025-04-02</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>PO-1003</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="n">
+        <v>71000</v>
+      </c>
+      <c r="I10" s="3" t="n">
+        <v>67500</v>
+      </c>
+      <c r="J10" s="3" t="n">
+        <v>3500</v>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
           <t>AMOUNT_MISMATCH</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
-        <is>
-          <t>Invoice amount 63720 does not match PO approved amount 54000.0. Difference: 9,720</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-07 18:52</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>INV-009.docx</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>INV-009</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>Tata Consultancy Services Ltd</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>Tata Consultancy Services Ltd</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>2025-04-02</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>PO-1003</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="n">
-        <v>83780</v>
-      </c>
-      <c r="I10" s="2" t="n">
-        <v>67500</v>
-      </c>
-      <c r="J10" s="2" t="n">
-        <v>16280</v>
-      </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="L10" s="3" t="inlineStr">
+        <is>
+          <t>Invoice amount 71000 does not match PO approved amount 67500.0. Difference: 3,500</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-07 19:48</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>INV-010.docx</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>INV-010</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Infosys Technologies Pvt Ltd</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Infosys Technologies Pvt Ltd</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>2025-05-10</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>PO-1006</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="n">
+        <v>61000</v>
+      </c>
+      <c r="I11" s="3" t="n">
+        <v>55000</v>
+      </c>
+      <c r="J11" s="3" t="n">
+        <v>6000</v>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
         <is>
           <t>AMOUNT_MISMATCH</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
-        <is>
-          <t>Invoice amount 83780 does not match PO approved amount 67500.0. Difference: 16,280</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-07 18:52</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>INV-010.docx</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>INV-010</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>Infosys Technologies Pvt Ltd</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>Infosys Technologies Pvt Ltd</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>2025-05-10</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>PO-1006</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="n">
-        <v>71980</v>
-      </c>
-      <c r="I11" s="2" t="n">
-        <v>55000</v>
-      </c>
-      <c r="J11" s="2" t="n">
-        <v>16980</v>
-      </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="L11" s="3" t="inlineStr">
+        <is>
+          <t>Invoice amount 61000 does not match PO approved amount 55000.0. Difference: 6,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-07 19:48</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>INV-011.docx</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>INV-011</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>HCL Technologies Limited</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>HCL Technologies Limited</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>2025-04-10</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>PO-1011</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="n">
+        <v>95000</v>
+      </c>
+      <c r="I12" s="3" t="n">
+        <v>99500</v>
+      </c>
+      <c r="J12" s="3" t="n">
+        <v>-4500</v>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
         <is>
           <t>AMOUNT_MISMATCH</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
-        <is>
-          <t>Invoice amount 71980 does not match PO approved amount 55000.0. Difference: 16,980</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-07 18:52</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>INV-011.docx</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>INV-011</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="L12" s="3" t="inlineStr">
+        <is>
+          <t>Invoice amount 95000 does not match PO approved amount 99500.0. Difference: 4,500</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>2026-06-07 19:48</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>INV-012.xlsx</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>INV-012</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Mphasis Software Services</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Mphasis Software Services</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>2025-05-20</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>PO-1014</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="n">
+        <v>82000</v>
+      </c>
+      <c r="I13" s="3" t="n">
+        <v>78000</v>
+      </c>
+      <c r="J13" s="3" t="n">
+        <v>4000</v>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>AMOUNT_MISMATCH</t>
+        </is>
+      </c>
+      <c r="L13" s="3" t="inlineStr">
+        <is>
+          <t>Invoice amount 82000 does not match PO approved amount 78000.0. Difference: 4,000</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-07 19:48</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>INV-013.xlsx</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>INV-013</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Wipro Digital Solutions</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="n"/>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>2025-04-22</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>PO-9901</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="n">
+        <v>48000</v>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J14" s="4" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K14" s="4" t="inlineStr">
+        <is>
+          <t>PO_NOT_FOUND</t>
+        </is>
+      </c>
+      <c r="L14" s="4" t="inlineStr">
+        <is>
+          <t>PO number 'PO-9901' not found in PO master.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-07 19:48</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>INV-014.xlsx</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>INV-014</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>HCL Technologies Limited</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>HCL Technologies Limited</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>2025-04-10</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>PO-1011</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="n">
-        <v>112100</v>
-      </c>
-      <c r="I12" s="2" t="n">
-        <v>99500</v>
-      </c>
-      <c r="J12" s="2" t="n">
-        <v>12600</v>
-      </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>AMOUNT_MISMATCH</t>
-        </is>
-      </c>
-      <c r="L12" s="2" t="inlineStr">
-        <is>
-          <t>Invoice amount 112100 does not match PO approved amount 99500.0. Difference: 12,600</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-07 18:52</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>INV-012.xlsx</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>INV-012</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>Mphasis Software Services</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>Mphasis Software Services</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>2025-05-20</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>PO-1014</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="n">
-        <v>96760</v>
-      </c>
-      <c r="I13" s="2" t="n">
-        <v>78000</v>
-      </c>
-      <c r="J13" s="2" t="n">
-        <v>18760</v>
-      </c>
-      <c r="K13" s="2" t="inlineStr">
-        <is>
-          <t>AMOUNT_MISMATCH</t>
-        </is>
-      </c>
-      <c r="L13" s="2" t="inlineStr">
-        <is>
-          <t>Invoice amount 96760 does not match PO approved amount 78000.0. Difference: 18,760</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>2026-06-07 18:52</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>INV-013.xlsx</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>INV-013</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>Wipro Digital Solutions</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="n"/>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>2025-04-22</t>
-        </is>
-      </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>PO-9901</t>
-        </is>
-      </c>
-      <c r="H14" s="3" t="n">
-        <v>56640</v>
-      </c>
-      <c r="I14" s="3" t="inlineStr">
+      <c r="E15" s="4" t="n"/>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>2025-05-05</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>PO-9902</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="n">
+        <v>21000</v>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="J14" s="3" t="inlineStr">
+      <c r="J15" s="4" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="K14" s="3" t="inlineStr">
+      <c r="K15" s="4" t="inlineStr">
         <is>
           <t>PO_NOT_FOUND</t>
         </is>
       </c>
-      <c r="L14" s="3" t="inlineStr">
-        <is>
-          <t>PO number 'PO-9901' not found in PO master.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>2026-06-07 18:52</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>INV-014.xlsx</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>INV-014</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>HCL Technologies Limited</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="n"/>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>2025-05-05</t>
-        </is>
-      </c>
-      <c r="G15" s="3" t="inlineStr">
-        <is>
-          <t>PO-9902</t>
-        </is>
-      </c>
-      <c r="H15" s="3" t="n">
-        <v>24780</v>
-      </c>
-      <c r="I15" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="J15" s="3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K15" s="3" t="inlineStr">
-        <is>
-          <t>PO_NOT_FOUND</t>
-        </is>
-      </c>
-      <c r="L15" s="3" t="inlineStr">
+      <c r="L15" s="4" t="inlineStr">
         <is>
           <t>PO number 'PO-9902' not found in PO master.</t>
         </is>
@@ -1303,7 +1309,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>2026-06-07 18:52</t>
+          <t>2026-06-07 19:49</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1337,22 +1343,22 @@
         </is>
       </c>
       <c r="H16" s="2" t="n">
-        <v>38940</v>
+        <v>33000</v>
       </c>
       <c r="I16" s="2" t="n">
         <v>33000</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>5940</v>
+        <v>0</v>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>AMOUNT_MISMATCH</t>
+          <t>MATCH</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>Invoice amount 38940 does not match PO approved amount 33000.0. Difference: 5,940</t>
+          <t>Invoice matches PO record.</t>
         </is>
       </c>
     </row>

</xml_diff>